<commit_message>
updated charts for paper
</commit_message>
<xml_diff>
--- a/DATA/production_capacity_updated.xlsx
+++ b/DATA/production_capacity_updated.xlsx
@@ -1,36 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{5BC75AC5-5DFF-42F9-8F6A-B58AA24898A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7606249-FD6D-40C8-A63D-37B30004849B}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{5BC75AC5-5DFF-42F9-8F6A-B58AA24898A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7213EFCE-AC76-4D7C-B7F4-5EE5C8F055CC}"/>
   <bookViews>
-    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
   </bookViews>
   <sheets>
     <sheet name="vaccine-producer list" sheetId="8" r:id="rId1"/>
-    <sheet name="total_capacity_calcs" sheetId="7" r:id="rId2"/>
-    <sheet name="Prod_capacity_agg" sheetId="9" r:id="rId3"/>
-    <sheet name="Producers_short_name" sheetId="5" r:id="rId4"/>
-    <sheet name="Medium_Capacity" sheetId="6" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="10" r:id="rId2"/>
+    <sheet name="total_capacity_calcs" sheetId="7" r:id="rId3"/>
+    <sheet name="Prod_capacity_agg" sheetId="9" r:id="rId4"/>
+    <sheet name="Producers_short_name" sheetId="5" r:id="rId5"/>
+    <sheet name="Medium_Capacity" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Medium_Capacity!$A$1:$K$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Prod_capacity_agg!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">total_capacity_calcs!$A$229:$L$296</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Medium_Capacity!$A$1:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Prod_capacity_agg!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">total_capacity_calcs!$A$229:$L$296</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'vaccine-producer list'!$A$1:$R$54</definedName>
-    <definedName name="GAVI_countries" localSheetId="1">#REF!</definedName>
+    <definedName name="GAVI_countries" localSheetId="2">#REF!</definedName>
     <definedName name="GAVI_countries" localSheetId="0">#REF!</definedName>
     <definedName name="GAVI_countries">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029" concurrentCalc="0"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3627,6 +3628,106 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84531983-CF53-47CA-A5F1-954F5A577DF5}">
+  <dimension ref="D4:F19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>15</v>
+      </c>
+      <c r="E4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>100</v>
+      </c>
+      <c r="E5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>47</v>
+      </c>
+      <c r="E7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <v>58</v>
+      </c>
+      <c r="E8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <v>40</v>
+      </c>
+      <c r="E10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <v>40</v>
+      </c>
+      <c r="E12">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <v>100</v>
+      </c>
+      <c r="E14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D16">
+        <v>81</v>
+      </c>
+      <c r="E16">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D18">
+        <v>41</v>
+      </c>
+      <c r="E18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D19">
+        <f>SUM(D4:D18)</f>
+        <v>522</v>
+      </c>
+      <c r="E19">
+        <f>SUM(E4:E18)</f>
+        <v>555</v>
+      </c>
+      <c r="F19">
+        <f>D19/E19</f>
+        <v>0.94054054054054059</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7054496A-AF4B-4EC1-B368-49C550220A1C}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:L301"/>
@@ -14291,16 +14392,36 @@
     </filterColumn>
   </autoFilter>
   <mergeCells count="52">
-    <mergeCell ref="A187:A191"/>
-    <mergeCell ref="A192:A195"/>
-    <mergeCell ref="A196:A198"/>
-    <mergeCell ref="A199:A203"/>
-    <mergeCell ref="A164:A167"/>
-    <mergeCell ref="A168:A172"/>
-    <mergeCell ref="A173:A175"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A181"/>
-    <mergeCell ref="A182:A186"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A22:A26"/>
+    <mergeCell ref="A70:A74"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A45:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A69"/>
+    <mergeCell ref="A114:A118"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="A90:A94"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="A98:A100"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A113"/>
     <mergeCell ref="A161:A163"/>
     <mergeCell ref="A120:A122"/>
     <mergeCell ref="A123:A125"/>
@@ -14313,36 +14434,16 @@
     <mergeCell ref="A150:A152"/>
     <mergeCell ref="A153:A156"/>
     <mergeCell ref="A157:A160"/>
-    <mergeCell ref="A114:A118"/>
-    <mergeCell ref="A75:A76"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="A90:A94"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A98:A100"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="A70:A74"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A45:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A69"/>
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A22:A26"/>
+    <mergeCell ref="A187:A191"/>
+    <mergeCell ref="A192:A195"/>
+    <mergeCell ref="A196:A198"/>
+    <mergeCell ref="A199:A203"/>
+    <mergeCell ref="A164:A167"/>
+    <mergeCell ref="A168:A172"/>
+    <mergeCell ref="A173:A175"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A181"/>
+    <mergeCell ref="A182:A186"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -14350,7 +14451,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55228539-2602-4D9E-BF99-AB1A3FA50A1F}">
   <dimension ref="A1:W63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -18300,7 +18401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{770C77AF-CB50-4854-8654-5465FF2CEF2B}">
   <dimension ref="B2:T19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -18575,7 +18676,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DF17EB8-02F1-485E-9D81-51CF2F0BE0EA}">
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>